<commit_message>
docs: rewrite README around verified behaviour; regenerate sample outputs
- README covers quick start (no-key demo, Docker, live model), the actual architecture,
  design decisions, LLM modes, API, configuration, testing and known limitations.
  Unverified claims (sub-millisecond search, 100k SKUs, zero hallucination, cost
  reduction) are removed; evaluation numbers come with how to read them.
- evals/RESULTS.md: replay and offline evaluation reports.
- exports/ regenerated with 'make demo', including the new processing-audit sheet.
</commit_message>
<xml_diff>
--- a/exports/commerceops_operations_report.xlsx
+++ b/exports/commerceops_operations_report.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="email-classification" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="order-status" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="order-response" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inquiry-response" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="email-classification" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="order-status" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="order-response" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="inquiry-response" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="processing-audit" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +21,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,14 +419,18 @@
   </sheetPr>
   <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>email ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
@@ -730,26 +723,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>email ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>product ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -938,16 +937,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>E017</t>
+          <t>E018</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>RSG8901</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -958,78 +957,38 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>E018</t>
+          <t>E019</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RSG8901</t>
+          <t>CBT8901</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>out of stock</t>
+          <t>created</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>E019</t>
+          <t>E023</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CBT8901</t>
+          <t>CGN2345</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D13" t="inlineStr">
-        <is>
-          <t>created</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>E022</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>UNKNOWN</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>out of stock</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>E023</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>CGN2345</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>5</v>
-      </c>
-      <c r="D15" t="inlineStr">
         <is>
           <t>out of stock</t>
         </is>
@@ -1048,14 +1007,18 @@
   </sheetPr>
   <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>email ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>response</t>
         </is>
@@ -1069,18 +1032,13 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Subject: Order Confirmation for Leather Bifold Wallets
-Dear Valued Customer,
-Thank you for reaching out and choosing our Leather Bifold Wallets for your boutique shop. We are thrilled to be a part of your new venture!
-I am pleased to confirm that your order for the remaining Leather Bifold Wallets has been successfully created. Here are the details of your order:
-- Leather Bifold Wallet (Product ID: LTH0976): 4 units
-Please note that these are the last units currently available in our inventory. Your order will be processed promptly, and you will receive a notification once it is shipped.
-If you have any further questions or need assistance with anything else, feel free to reach out. We are here to help and wish you great success with your boutique.
+          <t>Hello,
+Thank you for thinking of us for your new boutique! We have reserved all 4 remaining Leather Bifold Wallets (LTH0976) for you, and your order is now being prepared for shipment.
+We hope they find happy owners in your shop. If you would like to discuss larger quantities for future restocks, simply reply to this email.
 Warm regards,
-Aura Concierge
-Senior Customer Concierge
+The Aura Concierge Team
 Aura Fashion Atelier
-concierge@aurafashion.com</t>
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1092,16 +1050,13 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Subject: Your Vibrant Tote Order Confirmation
-Dear Jessica,
-Good morning! Thank you so much for reaching out and for sharing your love for tote bags with us. We completely agree—they're incredibly versatile and stylish!
-I'm delighted to confirm that your order for the Vibrant Tote (Product ID: VBT2345) has been successfully created. We have reserved 1 Vibrant Tote for you, and it will be on its way shortly.
-If you have any further questions or need assistance with anything else, please don't hesitate to let us know. We're here to help!
-Thank you for choosing us, and we hope you enjoy your new tote bag as much as your previous ones.
+          <t>Dear Jessica,
+Thank you for your order! We're happy to confirm 1 Vibrant Tote (VBT2345); it is now being prepared for shipment.
+It sounds like it will be in excellent company with your straw and nylon totes. Enjoy carrying it!
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1113,16 +1068,13 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Subject: Your Infinity Scarf Order Confirmation
-Dear Valued Customer,
-Thank you for choosing our brand for your wife's scarf collection. We are delighted to confirm that your order for the Infinity Scarves has been successfully created.
-Order Details:
-- Infinity Scarf (Product ID: SFT1098) - Quantity: 4
-We appreciate your business and are thrilled to be a part of your wife's collection. If you have any further questions or need assistance, please feel free to reach out.
+          <t>Hello,
+Thank you for your order! We're delighted to confirm 4 Infinity Scarves (SFT1098), and they are now being prepared for shipment.
+What a lovely addition to your wife's collection.
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1134,20 +1086,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Subject: Update on Your Order Request
-Dear Liz,
-Thank you for reaching out and considering our products for your holiday gift baskets. We appreciate your order and are here to assist you.
-I wanted to inform you that while we have successfully created your order for 2 pairs of Fuzzy Slippers, the Cable Knit Beanies are currently out of stock. We only have 2 Cable Knit Beanies available at the moment, instead of the 5 you requested.
-Here’s a summary of your order:
-- **Fuzzy Slippers (FZZ1098):** 2 pairs (Order Created)
-- **Cable Knit Beanie (CLF2109):** 0 available (Out of Stock)
-We apologize for any inconvenience this may cause. As an alternative, we can either send the 2 available Cable Knit Beanies or suggest similar styles that might suit your needs. Additionally, we expect to restock the Cable Knit Beanies soon, and I can notify you once they are available.
-Please let us know how you would like to proceed, and we will do our best to accommodate your preferences.
-Thank you for your understanding and patience.
+          <t>Dear Liz,
+Thank you for your order! Here is where it stands:
+- Fuzzy Slippers (FZZ1098) x 2: confirmed and being prepared for shipment.
+- Cable Knit Beanie (CLF2109) x 5: unfortunately we only have 2 in stock, so we couldn't reserve the 5 you asked for and nothing has been charged for them.
+For your gift baskets, the Chunky Knit Beanie (CHN0987, $22.00) or the Infinity Scarf (SFT1098, $28.00) could be lovely alternatives. We'd also be happy to let you know when the Cable Knit Beanie is back in stock.
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1159,17 +1106,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Subject: Your Versatile Scarf Order Confirmation
-Dear Valued Customer,
-Thank you for choosing our brand for your fashion needs! We are delighted to confirm that your order for the Versatile Scarf, which can be worn as a scarf, shawl, or headwrap, has been successfully created.
-Order Details:
-- Versatile Scarf: 1 piece
-We appreciate your business and are excited to have you as part of our fashion community. Your order will be processed shortly, and you will receive a notification once it has been shipped.
-If you have any further questions or need assistance, please do not hesitate to reach out.
+          <t>Hello,
+Thank you for your order! We're pleased to confirm 1 Versatile Scarf (VSC6789), the lightweight piece that can be worn as a scarf, shawl or headwrap. It is now being prepared for shipment.
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1181,14 +1123,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Subject: Your Order Confirmation - Retro Sunglasses
-Dear Valued Customer,
-Thank you for choosing our brand for your fashion needs! I'm delighted to confirm that your order for 1 pair of Retro Sunglasses (Product ID: RSG8901) has been successfully created.
-We appreciate your business and are excited for you to receive your new sunglasses. If you have any questions or need further assistance, please don't hesitate to reach out.
+          <t>Hello,
+Thank you for your order! We're happy to confirm 1 pair of Retro Sunglasses (RSG8901); they are now being prepared for shipment. Enjoy the sunshine!
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1200,16 +1140,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Subject: Your Order Confirmation - Slide Sandals
-Dear Marco,
-Thank you for choosing our brand for your summer footwear needs! I am pleased to confirm that your order for the following item has been successfully created:
-- Slide Sandals (Men's Shoes) - Quantity: 1
-We appreciate your purchase and are excited to be a part of your summer adventures. Your sandals will be on their way to you shortly.
-If you have any further questions or need assistance, please don't hesitate to reach out.
+          <t>Dear Marco,
+Thank you for your order! We're happy to confirm 1 pair of Slide Sandals (SLD7654) from our Men's Shoes collection; they are now being prepared for shipment, just in time for summer.
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1221,17 +1157,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Subject: Your Order Confirmation - Sleek Wallet
-Dear Johny,
-Thank you for your order with us!
-We are pleased to confirm that your order for the following item has been successfully created:
-- Sleek Wallet: Quantity 1
-Your order is being processed and will be dispatched shortly. You can expect to receive a shipping confirmation email with tracking details once your order is on its way.
-If you have any questions or need further assistance, please feel free to reach out.
-Thank you for choosing us for your fashion needs!
+          <t>Dear Johny,
+Thank you for your order! We're pleased to confirm 1 Sleek Wallet (SWL2345); it is now being prepared for shipment.
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1243,17 +1174,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Subject: Update on Your Order Request
-Dear Valued Customer,
-Thank you for reaching out to us and expressing interest in our popular item. We truly appreciate your enthusiasm for our products.
-Unfortunately, the item you requested is currently out of stock due to high demand. We understand how disappointing this can be, and we apologize for any inconvenience caused.
-We are actively working to restock this item and anticipate having it available again soon. In the meantime, we would be happy to suggest similar products that are currently in stock or notify you once the item becomes available again.
-Please let us know how you would like to proceed, and we will do our best to assist you.
-Thank you for your understanding and patience.
+          <t>Hello,
+Thank you for wanting to place an order! We'd love to help, but we couldn't tell which item you mean. Could you reply with the product name or its product ID (three letters followed by four digits, as shown on the product page) and how many you'd like? We'll confirm availability right away.
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1265,16 +1191,13 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Subject: Update on Your Order Request
-Dear Valued Customer,
-Thank you for reaching out to us with your interest in purchasing the Retro Sunglasses (RSG8901). We truly appreciate your enthusiasm for our products.
-Unfortunately, I must inform you that the Retro Sunglasses are currently out of stock, and we are unable to fulfill your request for 2 pairs at this time. We apologize for any inconvenience this may cause.
-As an alternative, we would be happy to notify you once the item is back in stock or assist you in selecting a similar style from our current collection. Please let us know how you would like to proceed, and we will do our best to accommodate your needs.
-Thank you for your understanding and patience. We look forward to assisting you further.
+          <t>Hello,
+Thank you for your order. Unfortunately the Retro Sunglasses (RSG8901) are currently out of stock, so we couldn't reserve the 2 pairs you requested and nothing has been charged.
+If you're shopping for summer accessories, the Bucket Hat (BKR0123, $39.99) is available now. We'd be happy to notify you as soon as the Retro Sunglasses are back in stock.
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1286,16 +1209,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Subject: Your Order Confirmation
-Dear Valued Customer,
-Thank you so much for your kind words and for your continued trust in our brand! We are thrilled to hear that you loved the quality of our Fuzzy Slippers, and we are confident that you will be equally impressed with your new purchase.
-I am pleased to confirm that your order for the Chelsea Boots [CBT 89 01] has been successfully created. We have reserved 1 pair for you, and it will be on its way shortly.
-Should you decide to go ahead with the Retro sunglasses in the future, please feel free to reach out. We would be delighted to assist you with that order as well.
-Thank you once again for choosing us. If you have any further questions or need assistance, please don't hesitate to contact us.
+          <t>Hello,
+Thank you so much for the kind words, and we're thrilled you're enjoying your Fuzzy Slippers! We're happy to confirm 1 pair of Chelsea Boots (CBT8901); your order is now being prepared for shipment.
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1307,17 +1226,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Subject: Update on Your Order Request
-Dear Monica,
-Thank you for reaching out and for your enthusiasm about our latest collection! We truly appreciate your support and excitement.
-I understand you're interested in purchasing three of our geometric pattern bags in the darker shade. Unfortunately, it seems that the specific item you are interested in is currently out of stock. We apologize for any inconvenience this may cause.
-As an alternative, I would recommend checking out our other available designs in the geometric collection, which might catch your interest. Additionally, we anticipate restocking the darker shade soon, and I can notify you as soon as it becomes available if you wish.
-Please let me know how you would like to proceed, and I will be more than happy to assist you further.
-Thank you for your understanding and patience.
+          <t>Dear Monica,
+Thank you for your enthusiasm, and we're excited you'd like to order! We couldn't match the geometric-pattern bags you saw to a specific product, so we haven't reserved anything yet. Could you reply with the product name or product ID (three letters followed by four digits) and the colour you'd like? We'll confirm availability for your 3 bags right away. Payment is handled securely at checkout, so there's no need to send cash.
 Warm regards,
-Aura Concierge
-Aura Customer Experience Concierge
-Aura Fashion Atelier</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1329,21 +1243,13 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Subject: Update on Your Order Request for Cargo Pants
-Dear Valued Customer,
-Thank you for reaching out and for your interest in our CGN2345 Cargo Pants. We truly appreciate your enthusiasm and commitment to our brand.
-Upon reviewing your order request, I regret to inform you that we currently have insufficient stock to fulfill your order of 5 Cargo Pants. At this moment, we only have 2 units available in our inventory.
-Here are a few options you might consider:
-1. **Proceed with Available Stock**: We can process an order for the 2 Cargo Pants currently in stock.
-2. **Wait for Restock**: We can notify you as soon as the additional stock becomes available.
-3. **Explore Alternatives**: If you're interested, I can assist you in finding similar items that are in stock.
-Please let us know how you would like to proceed, and we will be more than happy to assist you further.
-Thank you for your understanding and patience. We look forward to helping you complete your purchase.
+          <t>Hello,
+Thank you for your decision. Unfortunately we only have 2 Cargo Pants (CGN2345) in stock, so we couldn't reserve all 5 and nothing has been charged.
+If you'd like a similar style that is available now, consider the Corduroy Pants (CRD3210, $65.00) or the Overalls Jumpsuit (OVR3210, $55.99). We'd also be glad to let you know when the Cargo Pants are restocked.
 Warm regards,
-Aura Concierge
-Senior Customer Concierge
+The Aura Concierge Team
 Aura Fashion Atelier
-concierge@aurafashion.com</t>
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1360,14 +1266,18 @@
   </sheetPr>
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>email ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>response</t>
         </is>
@@ -1381,14 +1291,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hello David,
-Thank you for reaching out with your question about choosing the right bag for your work needs. Both the Leather Backpack (LTH1098) and the Leather Tote (LTH5432) are excellent choices, but they do have some differences that might help you decide.
-The **Leather Backpack** is priced at $43.99 and offers multiple compartments, including a padded laptop sleeve, which is ideal for securely carrying your laptop and organizing other documents or items. Its adjustable straps also provide comfort, making it a great option if you prefer carrying your items on your back.
-On the other hand, the **Leather Tote** is priced at $28.00 and features a spacious interior with multiple pockets. This bag is perfect if you prefer a more traditional carry style with sturdy handles, and it offers ample space for documents and other essentials.
-If organizational pockets are a priority, the Leather Backpack might be more suitable due to its multiple compartments and dedicated laptop sleeve. However, if you prefer a more classic tote style, the Leather Tote also provides good organizational features with its multiple pockets.
-I hope this helps you make a decision! If you have any more questions, feel free to ask.
-Best regards,
-Aura Concierge</t>
+          <t>Dear David,
+Both are excellent choices for carrying a laptop and documents to work:
+- Leather Backpack (LTH1098), $43.99, all seasons: multiple compartments, a padded laptop sleeve and adjustable straps. It offers the most built-in organization and protection for your laptop.
+- Leather Tote (LTH5432), $28.00, all seasons: full-grain leather with a spacious interior and multiple pockets. It has a more polished look but no dedicated laptop sleeve is listed.
+If organization and laptop protection come first, the Leather Backpack is the stronger fit. If you prefer a shoulder-carry style, the Leather Messenger Bag (LTH2109, $37.99) is a good middle ground with a spacious main compartment and multiple pockets.
+Warm regards,
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1400,11 +1311,13 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Good day,
-Thank you for your inquiry about the CSH1098 Cozy Shawl. This shawl is indeed designed to be versatile, allowing it to function both as a shawl and a lightweight blanket. It is knitted from soft, warm yarn, making it suitable for use as a lap blanket, especially during chilly evenings. At $22, it offers good quality for its price, providing comfort and warmth. It would make a thoughtful gift for your grandmother, offering her both style and coziness.
-If you have any more questions or need further assistance, feel free to reach out.
-Best regards,
-Aura Concierge</t>
+          <t>Hello,
+The Cozy Shawl (CSH1098, $22.00, Fall and Winter) is knitted from soft, warm yarn and is designed to be worn as a shawl, a scarf or a lightweight blanket. That makes it well suited as a light lap blanket for chilly evenings. It is not described as a heavy, thick throw, so for a warmer, more substantial feel it works best layered.
+Our catalog doesn't list the exact fibre content, so we can't promise a specific material. It is in stock and would make a thoughtful gift for your grandmother.
+Warm regards,
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1416,12 +1329,13 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hi Sam,
-Thank you for reaching out! The CBT8901 Chelsea Boots would be a great choice for the colder months, especially since they're designed for both Fall and Winter. With their sleek leather construction and sturdy lug sole, they’re perfect for elevating your casual looks with a modern, edgy touch.
-If you're planning to wait until Fall to place your order, that's a smart move as these boots are ideal for the season. In case you’re considering other options, our Rugged Boots (RBT0123) are also a fantastic choice for Fall and Winter, offering both style and functionality for outdoor adventures or city explorations.
-Feel free to reach out if you have any more questions or need further assistance!
-Best regards,
-Aura Concierge</t>
+          <t>Dear Sam,
+Thank you for letting us know you have your eye on the Chelsea Boots (CBT8901). They are $65.00, made for Fall and Winter, with sleek leather construction, elastic side panels and a sturdy lug sole, ideal for the colder months.
+They are currently in stock, but quantities are limited, so we can't guarantee availability in the Fall. If you'd like something more rugged for wet weather, the Waterproof Boots (WTR7654, $51.00) have a fleece lining and a lug sole for traction. Just reply when you're ready to order.
+Warm regards,
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1434,10 +1348,12 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>Hola,
-Gracias por tu consulta sobre el gorro de punto grueso DHN0987. El catálogo incluye nuestro **Gorro de punto grueso (CHN0987)**, tejido con hilo grueso y cálido, con un ajuste holgado y estilo rústico para protegerte del frío en otoño e invierno. Su precio es de $22.00.
-Si tienes más preguntas sobre las tallas o materiales, no dudes en escribirnos.
+Gracias por tu pregunta sobre el Gorro de punto grueso (Chunky Knit Beanie, CHN0987). Está tejido con un hilo grueso y acogedor, y nuestro catálogo no especifica la composición exacta de la fibra. Es una prenda pensada para otoño e invierno, con un ajuste holgado y amplio que mantiene la cabeza bien abrigada, así que es una buena opción para el frío.
+Cuesta $22.00 y actualmente está disponible. Si buscas completar el conjunto, el Cozy Sweater (CSW6789, $48.00) también es ideal para otoño e invierno.
 Saludos cordiales,
-Aura Concierge</t>
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1449,11 +1365,13 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hi there,
-Thank you for reaching out with your question about the RSG8901 Retro Sunglasses. These sunglasses are designed to evoke a nostalgic vibe reminiscent of the 1960s. They are perfect for adding a touch of vintage flair to your spring and summer outfits, whether you're heading to the beach or taking a stroll through the city.
-If you have any more questions or need further assistance, feel free to ask!
-Best regards,
-Aura Concierge</t>
+          <t>Hello,
+Thank you for your curiosity about the Retro Sunglasses (RSG8901, $26.99, Spring and Summer). Our catalog describes them as vintage-inspired shades with a cool, nostalgic vibe, but it doesn't name a specific decade, so we'd rather not guess between the 1950s and 1960s.
+If you enjoy that retro look, the Clog Sandals (CLG4567, $48.00) share the same throwback spirit for spring and summer.
+Warm regards,
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1466,11 +1384,15 @@
       <c r="B7" t="inlineStr">
         <is>
           <t>Hello,
-Thank you for reaching out and sharing your experience with our leather briefcase. I'm glad to hear you enjoyed it until the strap broke. For a new work bag, considering your preference for something slightly smaller, I recommend our **Leather Messenger Bag** (Product ID: LTH2109). It's crafted from premium, full-grain leather and offers a spacious main compartment, multiple pockets, and an adjustable strap for comfort. It's a timeless choice suitable for work, travel, or everyday use, priced at $37.99.
-If you're open to exploring other styles, our **Leather Tote** (Product ID: LTH5432) is another excellent option. It's slightly more compact and versatile, perfect for work or running errands, priced at $28.00.
-I hope this helps you find the perfect replacement. If you have any more questions or need further assistance, feel free to ask. Enjoy planning your anniversary dinner!
-Best regards,
-Aura Concierge</t>
+Sorry to hear the strap on your briefcase gave out after so much use. Here are some work-friendly options:
+- Leather Messenger Bag (LTH2109), $37.99: premium full-grain leather, a spacious main compartment, multiple pockets and an adjustable strap. The closest match to a briefcase-style carry.
+- Leather Tote (LTH5432), $28.00: full-grain leather with a spacious interior and multiple pockets, a slightly more relaxed silhouette.
+- Leather Backpack (LTH1098), $43.99: multiple compartments and a padded laptop sleeve if you carry a laptop.
+Our catalog doesn't list exact dimensions, so let us know what size your previous briefcase was and we can help you compare.
+Warm regards,
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1482,13 +1404,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Good morning,
-Thank you for reaching out with your thoughtful anniversary gift idea for Thomas. Based on your description, I recommend the **Leather Messenger Bag (Product ID: LTH2109)**. This bag is both stylish and practical, making it an excellent choice for his professional office environment as well as his outdoor weekend activities.
-The messenger bag is crafted from premium, full-grain leather, ensuring durability and a timeless look that suits all seasons. It features a spacious main compartment and multiple pockets, providing ample space for work essentials during the week and outdoor gear on weekends. The adjustable strap adds comfort, making it versatile for different settings.
-At $37.99, it offers great value for a multifunctional bag that seamlessly transitions from the office to the outdoors.
-Please let me know if you have any further questions or need assistance with your purchase.
-Best regards,
-Aura Concierge</t>
+          <t>Hello,
+What a thoughtful anniversary gift. For someone who goes from the office during the week to the trails on weekends, these stand out:
+- Leather Backpack (LTH1098), $43.99: premium leather with multiple compartments, a padded laptop sleeve and adjustable straps. Polished enough for work and comfortable for a hike.
+- Leather Messenger Bag (LTH2109), $37.99: full-grain leather, a spacious main compartment and an adjustable strap. A classic office choice.
+- Chic Crossbody (CCB6789), $35.00: compact with multiple compartments and adjustable straps, handy for lighter outdoor days.
+For the best of both worlds, we'd suggest the Leather Backpack.
+Warm regards,
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1500,12 +1425,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hello Claire,
-Thank you for reaching out! I have a lovely option that fits your preferences for a summer wedding guest dress. Consider our **Floral Maxi Dress**. It's designed for spring and summer, offering a breezy and lightweight feel that's perfect for an outdoor ceremony. The dress features a vibrant floral pattern and a flattering silhouette that flows gracefully, ensuring comfort without compromising style. It's priced at $56.0, and currently, you can enjoy a 20% discount.
-As for a travel bag, our **Leather Messenger Bag** could be an excellent choice. It's versatile for all seasons and crafted from premium full-grain leather, making it both stylish and functional for your travel needs. It’s priced at $37.99.
-I hope these options meet your needs for the wedding and your travels. If you have any more questions or need further assistance, feel free to ask!
-Best regards,
-Aura Concierge</t>
+          <t>Dear Claire,
+Thank you for sharing what you're looking for. In our current catalog we don't have a dress that matches all your wishes for an outdoor summer wedding: the Ribbed Bodycon Dress (RBB5432, $48.99, Spring to Fall) is form-fitting, and the Sweater Dress (SWT8765, $63.00) is a Winter piece, so neither is quite what you described.
+For travel, the Leather Messenger Bag (LTH2109, $37.99) offers a spacious main compartment, multiple pockets and an adjustable strap.
+If you can share your size and colour preferences, we'd be glad to let you know when new dresses arrive.
+Warm regards,
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1517,11 +1444,13 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hello Antonio,
-Thank you for reaching out. The Saddle Bag is priced at $39.00. It is designed for all seasons, making it a suitable choice for the spring season. This bag offers a vintage charm with its classic saddle shape and minimalist design, perfect for adding a retro flair to your spring outfits.
-If you have any more questions or need further assistance, feel free to ask!
-Best regards,  
-Aura Concierge</t>
+          <t>Dear Antonio,
+The Saddle Bag (SDE2345) is $39.00 and is an all-season piece, so it's a great choice for spring. It's a compact crossbody with a classic saddle shape and a minimalist design.
+Please note that stock is limited. If you'd like something with a little more boho flair for spring and summer, the Fringe Crossbody (FRP6789, $67.00) is another lovely option.
+Warm regards,
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
         </is>
       </c>
     </row>
@@ -1533,13 +1462,1510 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Thank you for reaching out and for being a valued customer with such a great taste in vintage items! I'm glad to hear that your previous purchases fit your style perfectly.
-Regarding your inquiry about winter hats, we offer two classic options: our **Chunky Knit Beanie (CHN0987)** priced at $22.00, crafted from thick cozy yarn for cold weather, and our **Cable Knit Beanie (CLF2109)** at $16.00, knitted from premium wool. Both provide warmth and vintage charm.
-If you have any other questions or need further styling assistance, feel free to let me know.
-Best regards,  
-Aura Concierge  
-Customer Experience Concierge</t>
-        </is>
+          <t>Hello,
+We're so glad your vintage pieces suit your style! For winter headwear with the same retro feel, we recommend the Corduroy Bucket Hat (CBY6789, $28.00, Fall and Winter), made from soft corduroy with a relaxed bucket silhouette. It would pair nicely with your Corduroy Pants.
+If you'd like more cold-weather vintage flair, the Ski Sweater (SKR3210, $57.00, Winter) has a chunky knit and a bold retro-inspired pattern.
+Warm regards,
+The Aura Concierge Team
+Aura Fashion Atelier
+concierge@aurafashion.com | +1 (800) 555-2872</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>email ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>customer name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>order lines</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>unresolved mentions</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>context products</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>guardrail flags</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>degraded</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>degraded reasons</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>llm calls</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>replayed calls</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>prompt tokens</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>completion tokens</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>latency ms</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>LTH0976</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>6</v>
+      </c>
+      <c r="R2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Jessica</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>VBT2345</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>6</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>LTH1098, LTH5432, QTP5432, LTH2109, SBP4567, VBT2345</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="b">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SFT1098</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="b">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>35</v>
+      </c>
+      <c r="R5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>CSH1098, VSC6789, CSW6789, CCG8901, SFT1098</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>8</v>
+      </c>
+      <c r="R6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>CBT8901, RBT0123, SNB4321, WTR7654, CHK8901</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>17</v>
+      </c>
+      <c r="R7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Liz</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>CLF2109, FZZ1098, CHN0987, SFT1098</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>8</v>
+      </c>
+      <c r="R8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>E008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>VSC6789</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>34</v>
+      </c>
+      <c r="R9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>E009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>es</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>CHN0987, CSW6789, CPJ2345, CHL4567, RBT0123</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="n">
+        <v>2</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>34</v>
+      </c>
+      <c r="R10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>E010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>RSG8901</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="b">
+        <v>0</v>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N11" t="n">
+        <v>3</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>60</v>
+      </c>
+      <c r="R11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>E011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>RSG8901, DJN8901, CLG4567, RGD7654, CRD3210</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="b">
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" t="n">
+        <v>2</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>22</v>
+      </c>
+      <c r="R12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LTH2109, CBG9876, LTH5432, LTH1098, QTP5432</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="b">
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" t="n">
+        <v>2</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>41</v>
+      </c>
+      <c r="R13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>E013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Marco</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>SLD7654</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="b">
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" t="n">
+        <v>3</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>21</v>
+      </c>
+      <c r="R14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>E014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Johny</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>SWL2345</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="n">
+        <v>3</v>
+      </c>
+      <c r="N15" t="n">
+        <v>3</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>44</v>
+      </c>
+      <c r="R15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>E015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>QTP5432, CCB6789, LTH2109, LTH1098</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="b">
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" t="n">
+        <v>2</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>31</v>
+      </c>
+      <c r="R16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>E016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Claire</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>SWT8765, LTH2109, RBB5432, RCS0123</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>30</v>
+      </c>
+      <c r="R17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>E017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>needs_clarification</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>that popular item</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>3</v>
+      </c>
+      <c r="N18" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>36</v>
+      </c>
+      <c r="R18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>E018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>RSG8901, BKR0123, CPN3210</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="b">
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" t="n">
+        <v>3</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>34</v>
+      </c>
+      <c r="R19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>E019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>CBT8901</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="b">
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" t="n">
+        <v>3</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>40</v>
+      </c>
+      <c r="R20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>E020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Antonio</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>SDE2345, FRP6789, CBG9876, LTH2109, CCB6789</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="b">
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>2</v>
+      </c>
+      <c r="N21" t="n">
+        <v>2</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>27</v>
+      </c>
+      <c r="R21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>E021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>product inquiry</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>SDE2345, DJN8901, RGD7654, CRD3210, FZV1098, SKR3210, BKR0123, CBY6789</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="b">
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>2</v>
+      </c>
+      <c r="N22" t="n">
+        <v>2</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>46</v>
+      </c>
+      <c r="R22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>E022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>needs_clarification</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Monica</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>bags with geometric patterns</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="b">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>3</v>
+      </c>
+      <c r="N23" t="n">
+        <v>3</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>23</v>
+      </c>
+      <c r="R23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>order request</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>CGN2345, CRD3210, OVR3210</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="b">
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>3</v>
+      </c>
+      <c r="N24" t="n">
+        <v>3</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>30</v>
+      </c>
+      <c r="R24" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>